<commit_message>
Actualizacion automatica 2026-09-14 18:31 UTC
</commit_message>
<xml_diff>
--- a/data/50001497 - XEMORTIZ IMMSA STA BBR.xlsx
+++ b/data/50001497 - XEMORTIZ IMMSA STA BBR.xlsx
@@ -181,160 +181,160 @@
     <t>Ingenieria de servicio:,ot 4196 - 4197-4198 Palatizado y  Embalaje</t>
   </si>
   <si>
+    <t>Tarea en curso</t>
+  </si>
+  <si>
+    <t>1213193408378967</t>
+  </si>
+  <si>
+    <t>Ingenieria Jefe de proyecto:</t>
+  </si>
+  <si>
+    <t>Ingenieria Detalle,Ingenieria basica Rodete,Ingenieria Basica Motor,Analisis de costeo</t>
+  </si>
+  <si>
+    <t>1213193408378968</t>
+  </si>
+  <si>
+    <t>Ingenieria Basica Motor</t>
+  </si>
+  <si>
+    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta motor</t>
+  </si>
+  <si>
+    <t>1213249277752961</t>
+  </si>
+  <si>
+    <t>Ingenieria basica Rodete</t>
+  </si>
+  <si>
+    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta nucleo rodete,propuesta alabes</t>
+  </si>
+  <si>
+    <t>1213249277752962</t>
+  </si>
+  <si>
+    <t>Ingenieria Detalle</t>
+  </si>
+  <si>
+    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,Propuesta sensores y accesorios,propuesta compras a codigo // aprovisionamiento,Planos Preliminar</t>
+  </si>
+  <si>
+    <t>1213249277752963</t>
+  </si>
+  <si>
+    <t>Analisis de costeo</t>
+  </si>
+  <si>
+    <t>Ingenieria Basica Motor,Ingenieria Detalle,Ingenieria basica Rodete</t>
+  </si>
+  <si>
+    <t>Ingenieria Jefe de proyecto:,Costos</t>
+  </si>
+  <si>
+    <t>1213249277752964</t>
+  </si>
+  <si>
+    <t>Propuesta compras:</t>
+  </si>
+  <si>
+    <t>propuesta motor,propuesta alabes,propuesta tableros,propuesta nucleo rodete,Propuesta sensores y accesorios,propuesta compras a codigo // aprovisionamiento</t>
+  </si>
+  <si>
+    <t>1213249277752965</t>
+  </si>
+  <si>
+    <t>propuesta motor</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC motor OT 4196</t>
+  </si>
+  <si>
+    <t>1213249277752966</t>
+  </si>
+  <si>
+    <t>propuesta alabes</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC Alabe</t>
+  </si>
+  <si>
+    <t>1213249277752967</t>
+  </si>
+  <si>
+    <t>propuesta tableros</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC Tableros</t>
+  </si>
+  <si>
+    <t>1213249277752968</t>
+  </si>
+  <si>
+    <t>propuesta nucleo rodete</t>
+  </si>
+  <si>
+    <t>NATALYA ESPINOZA</t>
+  </si>
+  <si>
+    <t>nespinoza@zitron.com</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC Rodete</t>
+  </si>
+  <si>
+    <t>1213249277752969</t>
+  </si>
+  <si>
+    <t>Propuesta sensores y accesorios</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC Sensores y accesorios</t>
+  </si>
+  <si>
+    <t>1213249277752970</t>
+  </si>
+  <si>
+    <t>propuesta compras a codigo // aprovisionamiento</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC materiales</t>
+  </si>
+  <si>
+    <t>1213249277752971</t>
+  </si>
+  <si>
+    <t>Compras:</t>
+  </si>
+  <si>
+    <t>Tablero,Alabe,rodete,Motor OT 4196,Materiales a codigo // compras locales aprovisionamientomiento,Sensores y accesorios</t>
+  </si>
+  <si>
+    <t>1213249277752972</t>
+  </si>
+  <si>
+    <t>Alabe</t>
+  </si>
+  <si>
+    <t>Eliana</t>
+  </si>
+  <si>
+    <t>ecarico@zitron.com</t>
+  </si>
+  <si>
+    <t>Generación OC Alabe,Fabricación Alabe</t>
+  </si>
+  <si>
+    <t>1213249277752973</t>
+  </si>
+  <si>
+    <t>Generación OC Alabe</t>
+  </si>
+  <si>
+    <t>Fabricación Alabe,Alabe</t>
+  </si>
+  <si>
     <t>Tarea sin iniciar</t>
-  </si>
-  <si>
-    <t>1213193408378967</t>
-  </si>
-  <si>
-    <t>Ingenieria Jefe de proyecto:</t>
-  </si>
-  <si>
-    <t>Ingenieria Detalle,Ingenieria basica Rodete,Ingenieria Basica Motor,Analisis de costeo</t>
-  </si>
-  <si>
-    <t>1213193408378968</t>
-  </si>
-  <si>
-    <t>Ingenieria Basica Motor</t>
-  </si>
-  <si>
-    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta motor</t>
-  </si>
-  <si>
-    <t>1213249277752961</t>
-  </si>
-  <si>
-    <t>Ingenieria basica Rodete</t>
-  </si>
-  <si>
-    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta nucleo rodete,propuesta alabes</t>
-  </si>
-  <si>
-    <t>1213249277752962</t>
-  </si>
-  <si>
-    <t>Ingenieria Detalle</t>
-  </si>
-  <si>
-    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,Propuesta sensores y accesorios,propuesta compras a codigo // aprovisionamiento,Planos Preliminar</t>
-  </si>
-  <si>
-    <t>1213249277752963</t>
-  </si>
-  <si>
-    <t>Analisis de costeo</t>
-  </si>
-  <si>
-    <t>Ingenieria Basica Motor,Ingenieria Detalle,Ingenieria basica Rodete</t>
-  </si>
-  <si>
-    <t>Ingenieria Jefe de proyecto:,Costos</t>
-  </si>
-  <si>
-    <t>1213249277752964</t>
-  </si>
-  <si>
-    <t>Propuesta compras:</t>
-  </si>
-  <si>
-    <t>propuesta motor,propuesta alabes,propuesta tableros,propuesta nucleo rodete,Propuesta sensores y accesorios,propuesta compras a codigo // aprovisionamiento</t>
-  </si>
-  <si>
-    <t>1213249277752965</t>
-  </si>
-  <si>
-    <t>propuesta motor</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC motor OT 4196</t>
-  </si>
-  <si>
-    <t>1213249277752966</t>
-  </si>
-  <si>
-    <t>propuesta alabes</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC Alabe</t>
-  </si>
-  <si>
-    <t>Tarea en curso</t>
-  </si>
-  <si>
-    <t>1213249277752967</t>
-  </si>
-  <si>
-    <t>propuesta tableros</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC Tableros</t>
-  </si>
-  <si>
-    <t>1213249277752968</t>
-  </si>
-  <si>
-    <t>propuesta nucleo rodete</t>
-  </si>
-  <si>
-    <t>NATALYA ESPINOZA</t>
-  </si>
-  <si>
-    <t>nespinoza@zitron.com</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC Rodete</t>
-  </si>
-  <si>
-    <t>1213249277752969</t>
-  </si>
-  <si>
-    <t>Propuesta sensores y accesorios</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC Sensores y accesorios</t>
-  </si>
-  <si>
-    <t>1213249277752970</t>
-  </si>
-  <si>
-    <t>propuesta compras a codigo // aprovisionamiento</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC materiales</t>
-  </si>
-  <si>
-    <t>1213249277752971</t>
-  </si>
-  <si>
-    <t>Compras:</t>
-  </si>
-  <si>
-    <t>Tablero,Alabe,rodete,Motor OT 4196,Materiales a codigo // compras locales aprovisionamientomiento,Sensores y accesorios</t>
-  </si>
-  <si>
-    <t>1213249277752972</t>
-  </si>
-  <si>
-    <t>Alabe</t>
-  </si>
-  <si>
-    <t>Eliana</t>
-  </si>
-  <si>
-    <t>ecarico@zitron.com</t>
-  </si>
-  <si>
-    <t>Generación OC Alabe,Fabricación Alabe</t>
-  </si>
-  <si>
-    <t>1213249277752973</t>
-  </si>
-  <si>
-    <t>Generación OC Alabe</t>
-  </si>
-  <si>
-    <t>Fabricación Alabe,Alabe</t>
   </si>
   <si>
     <t>Baja</t>
@@ -1855,7 +1855,7 @@
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="5">
-        <v>46097.55431952546</v>
+        <v>46279.7521228125</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>45</v>
@@ -1967,7 +1967,7 @@
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="5">
-        <v>46246.741893645834</v>
+        <v>46279.7523291088</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>53</v>
@@ -2012,9 +2012,9 @@
         <v>46136</v>
       </c>
       <c r="S12" s="6">
-        <v>0</v>
-      </c>
-      <c r="T12" s="11" t="s">
+        <v>0.8</v>
+      </c>
+      <c r="T12" s="12" t="s">
         <v>56</v>
       </c>
       <c r="U12" s="11" t="s">
@@ -2511,7 +2511,7 @@
         <v>1</v>
       </c>
       <c r="T20" s="12" t="s">
-        <v>82</v>
+        <v>56</v>
       </c>
       <c r="U20" s="11" t="s">
         <v>32</v>
@@ -2519,7 +2519,7 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B21" s="8">
         <v>46065.866394571756</v>
@@ -2531,7 +2531,7 @@
         <v>46097.55438569444</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>26</v>
@@ -2564,7 +2564,7 @@
         <v>48</v>
       </c>
       <c r="P21" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="Q21" s="8">
         <v>46010</v>
@@ -2584,7 +2584,7 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B22" s="5">
         <v>46065.86639490741</v>
@@ -2596,16 +2596,16 @@
         <v>46223.81276079861</v>
       </c>
       <c r="E22" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G22" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="F22" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G22" s="6" t="s">
+      <c r="H22" s="6" t="s">
         <v>88</v>
-      </c>
-      <c r="H22" s="6" t="s">
-        <v>89</v>
       </c>
       <c r="I22" s="5">
         <v>46017</v>
@@ -2629,7 +2629,7 @@
         <v>64</v>
       </c>
       <c r="P22" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="Q22" s="5">
         <v>46017</v>
@@ -2649,7 +2649,7 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B23" s="8">
         <v>46065.86638537037</v>
@@ -2661,7 +2661,7 @@
         <v>46114.52306825231</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>26</v>
@@ -2694,7 +2694,7 @@
         <v>67</v>
       </c>
       <c r="P23" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="Q23" s="8">
         <v>46017</v>
@@ -2714,7 +2714,7 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B24" s="5">
         <v>46065.86638577546</v>
@@ -2726,16 +2726,16 @@
         <v>46223.812757314816</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G24" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="H24" s="6" t="s">
         <v>88</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>89</v>
       </c>
       <c r="I24" s="5">
         <v>46017</v>
@@ -2759,7 +2759,7 @@
         <v>67</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="Q24" s="5">
         <v>46017</v>
@@ -2779,7 +2779,7 @@
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B25" s="8">
         <v>46065.86638607639</v>
@@ -2791,7 +2791,7 @@
         <v>46233.63103746528</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>25</v>
@@ -2815,7 +2815,7 @@
         <v>26</v>
       </c>
       <c r="O25" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="P25" s="9" t="s">
         <v>26</v>
@@ -2832,7 +2832,7 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B26" s="5">
         <v>46065.86638636574</v>
@@ -2844,16 +2844,16 @@
         <v>46155.87591685185</v>
       </c>
       <c r="E26" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G26" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="F26" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G26" s="6" t="s">
+      <c r="H26" s="6" t="s">
         <v>102</v>
-      </c>
-      <c r="H26" s="6" t="s">
-        <v>103</v>
       </c>
       <c r="I26" s="5">
         <v>46030</v>
@@ -2871,13 +2871,13 @@
         <v>26</v>
       </c>
       <c r="N26" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="P26" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="Q26" s="5">
         <v>46030</v>
@@ -2897,7 +2897,7 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B27" s="8">
         <v>46065.866386678244</v>
@@ -2909,16 +2909,16 @@
         <v>46097.553490011574</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G27" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="H27" s="9" t="s">
         <v>102</v>
-      </c>
-      <c r="H27" s="9" t="s">
-        <v>103</v>
       </c>
       <c r="I27" s="8">
         <v>46030</v>
@@ -2936,13 +2936,13 @@
         <v>26</v>
       </c>
       <c r="N27" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O27" s="9" t="s">
         <v>80</v>
       </c>
       <c r="P27" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="Q27" s="9"/>
       <c r="R27" s="9"/>
@@ -2950,7 +2950,7 @@
         <v>0</v>
       </c>
       <c r="T27" s="11" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="U27" s="10" t="s">
         <v>108</v>
@@ -2976,10 +2976,10 @@
         <v>26</v>
       </c>
       <c r="G28" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="H28" s="6" t="s">
         <v>102</v>
-      </c>
-      <c r="H28" s="6" t="s">
-        <v>103</v>
       </c>
       <c r="I28" s="5">
         <v>46034</v>
@@ -2997,10 +2997,10 @@
         <v>26</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="P28" s="6" t="s">
         <v>111</v>
@@ -3011,7 +3011,7 @@
         <v>0</v>
       </c>
       <c r="T28" s="11" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="U28" s="10" t="s">
         <v>108</v>
@@ -3037,10 +3037,10 @@
         <v>26</v>
       </c>
       <c r="G29" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="H29" s="9" t="s">
         <v>102</v>
-      </c>
-      <c r="H29" s="9" t="s">
-        <v>103</v>
       </c>
       <c r="I29" s="8">
         <v>46021</v>
@@ -3058,13 +3058,13 @@
         <v>26</v>
       </c>
       <c r="N29" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="O29" s="9" t="s">
         <v>114</v>
       </c>
       <c r="P29" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="Q29" s="8">
         <v>46021</v>
@@ -3102,10 +3102,10 @@
         <v>26</v>
       </c>
       <c r="G30" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="H30" s="6" t="s">
         <v>102</v>
-      </c>
-      <c r="H30" s="6" t="s">
-        <v>103</v>
       </c>
       <c r="I30" s="5">
         <v>46021</v>
@@ -3126,7 +3126,7 @@
         <v>113</v>
       </c>
       <c r="O30" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P30" s="6" t="s">
         <v>117</v>
@@ -3137,7 +3137,7 @@
         <v>0</v>
       </c>
       <c r="T30" s="11" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="U30" s="10" t="s">
         <v>108</v>
@@ -3163,10 +3163,10 @@
         <v>26</v>
       </c>
       <c r="G31" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="H31" s="9" t="s">
         <v>102</v>
-      </c>
-      <c r="H31" s="9" t="s">
-        <v>103</v>
       </c>
       <c r="I31" s="8">
         <v>46030</v>
@@ -3198,7 +3198,7 @@
         <v>0</v>
       </c>
       <c r="T31" s="11" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="U31" s="10" t="s">
         <v>108</v>
@@ -3224,10 +3224,10 @@
         <v>26</v>
       </c>
       <c r="G32" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="H32" s="6" t="s">
         <v>102</v>
-      </c>
-      <c r="H32" s="6" t="s">
-        <v>103</v>
       </c>
       <c r="I32" s="5">
         <v>46030</v>
@@ -3245,13 +3245,13 @@
         <v>26</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="O32" s="6" t="s">
         <v>123</v>
       </c>
       <c r="P32" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="Q32" s="5">
         <v>46030</v>
@@ -3289,10 +3289,10 @@
         <v>26</v>
       </c>
       <c r="G33" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="H33" s="9" t="s">
         <v>102</v>
-      </c>
-      <c r="H33" s="9" t="s">
-        <v>103</v>
       </c>
       <c r="I33" s="8">
         <v>46030</v>
@@ -3313,7 +3313,7 @@
         <v>122</v>
       </c>
       <c r="O33" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="P33" s="9" t="s">
         <v>126</v>
@@ -3324,7 +3324,7 @@
         <v>0</v>
       </c>
       <c r="T33" s="11" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="U33" s="10" t="s">
         <v>108</v>
@@ -3350,10 +3350,10 @@
         <v>26</v>
       </c>
       <c r="G34" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="H34" s="6" t="s">
         <v>102</v>
-      </c>
-      <c r="H34" s="6" t="s">
-        <v>103</v>
       </c>
       <c r="I34" s="5">
         <v>46034</v>
@@ -3385,7 +3385,7 @@
         <v>0</v>
       </c>
       <c r="T34" s="11" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="U34" s="10" t="s">
         <v>108</v>
@@ -3411,10 +3411,10 @@
         <v>26</v>
       </c>
       <c r="G35" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="H35" s="9" t="s">
         <v>102</v>
-      </c>
-      <c r="H35" s="9" t="s">
-        <v>103</v>
       </c>
       <c r="I35" s="8">
         <v>46013</v>
@@ -3432,13 +3432,13 @@
         <v>26</v>
       </c>
       <c r="N35" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="O35" s="9" t="s">
         <v>132</v>
       </c>
       <c r="P35" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="Q35" s="8">
         <v>46013</v>
@@ -3476,10 +3476,10 @@
         <v>26</v>
       </c>
       <c r="G36" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="H36" s="6" t="s">
         <v>102</v>
-      </c>
-      <c r="H36" s="6" t="s">
-        <v>103</v>
       </c>
       <c r="I36" s="5">
         <v>46013</v>
@@ -3511,7 +3511,7 @@
         <v>0</v>
       </c>
       <c r="T36" s="11" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="U36" s="10" t="s">
         <v>108</v>
@@ -3537,10 +3537,10 @@
         <v>26</v>
       </c>
       <c r="G37" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="H37" s="9" t="s">
         <v>102</v>
-      </c>
-      <c r="H37" s="9" t="s">
-        <v>103</v>
       </c>
       <c r="I37" s="8">
         <v>46036</v>
@@ -3572,7 +3572,7 @@
         <v>0</v>
       </c>
       <c r="T37" s="11" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="U37" s="10" t="s">
         <v>108</v>
@@ -3598,10 +3598,10 @@
         <v>26</v>
       </c>
       <c r="G38" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="H38" s="6" t="s">
         <v>102</v>
-      </c>
-      <c r="H38" s="6" t="s">
-        <v>103</v>
       </c>
       <c r="I38" s="5">
         <v>46036</v>
@@ -3633,7 +3633,7 @@
         <v>0</v>
       </c>
       <c r="T38" s="11" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="U38" s="10" t="s">
         <v>108</v>
@@ -3680,13 +3680,13 @@
         <v>26</v>
       </c>
       <c r="N39" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="O39" s="9" t="s">
         <v>146</v>
       </c>
       <c r="P39" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="Q39" s="8">
         <v>46030</v>
@@ -3748,7 +3748,7 @@
         <v>143</v>
       </c>
       <c r="O40" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="P40" s="6" t="s">
         <v>149</v>
@@ -3759,7 +3759,7 @@
         <v>0</v>
       </c>
       <c r="T40" s="11" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="U40" s="10" t="s">
         <v>108</v>
@@ -3820,7 +3820,7 @@
         <v>0</v>
       </c>
       <c r="T41" s="11" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="U41" s="10" t="s">
         <v>108</v>
@@ -3867,13 +3867,13 @@
         <v>26</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="O42" s="6" t="s">
         <v>155</v>
       </c>
       <c r="P42" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="Q42" s="5">
         <v>46030</v>
@@ -3935,7 +3935,7 @@
         <v>154</v>
       </c>
       <c r="O43" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="P43" s="9" t="s">
         <v>159</v>
@@ -3946,7 +3946,7 @@
         <v>0</v>
       </c>
       <c r="T43" s="11" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="U43" s="10" t="s">
         <v>108</v>
@@ -4007,7 +4007,7 @@
         <v>0</v>
       </c>
       <c r="T44" s="11" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="U44" s="10" t="s">
         <v>108</v>
@@ -4058,7 +4058,7 @@
       <c r="R45" s="9"/>
       <c r="S45" s="9"/>
       <c r="T45" s="12" t="s">
-        <v>82</v>
+        <v>56</v>
       </c>
       <c r="U45" s="9"/>
     </row>
@@ -4186,7 +4186,7 @@
         <v>1</v>
       </c>
       <c r="T47" s="12" t="s">
-        <v>82</v>
+        <v>56</v>
       </c>
       <c r="U47" s="11" t="s">
         <v>32</v>
@@ -4314,7 +4314,7 @@
         <v>0</v>
       </c>
       <c r="T49" s="11" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="U49" s="11" t="s">
         <v>32</v>
@@ -5050,7 +5050,7 @@
         <v>0</v>
       </c>
       <c r="T61" s="12" t="s">
-        <v>82</v>
+        <v>56</v>
       </c>
       <c r="U61" s="11" t="s">
         <v>32</v>
@@ -5194,10 +5194,10 @@
         <v>26</v>
       </c>
       <c r="G64" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="H64" s="6" t="s">
         <v>88</v>
-      </c>
-      <c r="H64" s="6" t="s">
-        <v>89</v>
       </c>
       <c r="I64" s="5">
         <v>46127</v>
@@ -5259,10 +5259,10 @@
         <v>26</v>
       </c>
       <c r="G65" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="H65" s="9" t="s">
         <v>88</v>
-      </c>
-      <c r="H65" s="9" t="s">
-        <v>89</v>
       </c>
       <c r="I65" s="8">
         <v>46164</v>
@@ -5324,10 +5324,10 @@
         <v>26</v>
       </c>
       <c r="G66" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="H66" s="6" t="s">
         <v>88</v>
-      </c>
-      <c r="H66" s="6" t="s">
-        <v>89</v>
       </c>
       <c r="I66" s="5">
         <v>46149</v>
@@ -5387,10 +5387,10 @@
         <v>26</v>
       </c>
       <c r="G67" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="H67" s="9" t="s">
         <v>88</v>
-      </c>
-      <c r="H67" s="9" t="s">
-        <v>89</v>
       </c>
       <c r="I67" s="8">
         <v>46153</v>
@@ -5426,7 +5426,7 @@
         <v>1</v>
       </c>
       <c r="T67" s="12" t="s">
-        <v>82</v>
+        <v>56</v>
       </c>
       <c r="U67" s="11" t="s">
         <v>32</v>
@@ -5452,10 +5452,10 @@
         <v>26</v>
       </c>
       <c r="G68" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="H68" s="6" t="s">
         <v>88</v>
-      </c>
-      <c r="H68" s="6" t="s">
-        <v>89</v>
       </c>
       <c r="I68" s="5">
         <v>46146</v>
@@ -5515,10 +5515,10 @@
         <v>26</v>
       </c>
       <c r="G69" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="H69" s="9" t="s">
         <v>88</v>
-      </c>
-      <c r="H69" s="9" t="s">
-        <v>89</v>
       </c>
       <c r="I69" s="9"/>
       <c r="J69" s="8">
@@ -5552,7 +5552,7 @@
         <v>0</v>
       </c>
       <c r="T69" s="11" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="U69" s="11" t="s">
         <v>32</v>
@@ -5576,10 +5576,10 @@
         <v>26</v>
       </c>
       <c r="G70" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="H70" s="6" t="s">
         <v>88</v>
-      </c>
-      <c r="H70" s="6" t="s">
-        <v>89</v>
       </c>
       <c r="I70" s="6"/>
       <c r="J70" s="5">
@@ -5613,7 +5613,7 @@
         <v>0</v>
       </c>
       <c r="T70" s="11" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="U70" s="11" t="s">
         <v>32</v>
@@ -5721,7 +5721,7 @@
         <v>0</v>
       </c>
       <c r="T72" s="11" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="U72" s="11" t="s">
         <v>32</v>
@@ -5745,10 +5745,10 @@
         <v>26</v>
       </c>
       <c r="G73" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="H73" s="9" t="s">
         <v>88</v>
-      </c>
-      <c r="H73" s="9" t="s">
-        <v>89</v>
       </c>
       <c r="I73" s="8">
         <v>46174</v>
@@ -5784,7 +5784,7 @@
         <v>0</v>
       </c>
       <c r="T73" s="12" t="s">
-        <v>82</v>
+        <v>56</v>
       </c>
       <c r="U73" s="11" t="s">
         <v>32</v>
@@ -5845,7 +5845,7 @@
         <v>0</v>
       </c>
       <c r="T74" s="11" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="U74" s="11" t="s">
         <v>32</v>
@@ -5906,7 +5906,7 @@
         <v>0</v>
       </c>
       <c r="T75" s="11" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="U75" s="11" t="s">
         <v>32</v>
@@ -6016,7 +6016,7 @@
         <v>0</v>
       </c>
       <c r="T77" s="11" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="U77" s="11" t="s">
         <v>32</v>
@@ -6079,7 +6079,7 @@
         <v>0</v>
       </c>
       <c r="T78" s="11" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="U78" s="11" t="s">
         <v>32</v>

</xml_diff>